<commit_message>
Accept P14 single-device lifecycle and synchronize execution plan
</commit_message>
<xml_diff>
--- a/docs/project-plans/lamda_yun_一期计划_智能体执行版.xlsx
+++ b/docs/project-plans/lamda_yun_一期计划_智能体执行版.xlsx
@@ -1,20 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00_执行总览" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01_闭环计划" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02_验收卡" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03_启动与门禁" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_旧任务对照" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05_范围追溯" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06_执行实测" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07_原审阅索引" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08_模型分工与解锁" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09_执行记录" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10_当前包交接模板" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="11_多智能体并行" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="00_执行总览" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="01_闭环计划" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="02_验收卡" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="03_启动与门禁" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="04_旧任务对照" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="05_范围追溯" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="06_执行实测" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="07_原审阅索引" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="08_模型分工与解锁" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="09_执行记录" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="10_当前包交接模板" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="11_多智能体并行" sheetId="12" state="visible" r:id="rId12"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'01_闭环计划'!$A$5:$S$55</definedName>
@@ -1354,7 +1354,7 @@
     <row r="2" ht="25" customHeight="1">
       <c r="A2" s="45" t="inlineStr">
         <is>
-          <t>2026-09-09 智能体执行版｜当前验收=现有 OnePlus 9R b0644fb5 单机分阶段。Note9/10台/100模拟为后期扩展（非已通过、非删除）。网页高级模型定方案，本地模型实施，达到触发条件才升级诊断。原功能与安全门禁在当前机上仍须满足，不预估人力工期。</t>
+          <t>2026-09-10 智能体执行版｜当前验收=现有 OnePlus 9R b0644fb5 单机分阶段。Note9/10台/100模拟为后期扩展（非已通过、非删除）。网页高级模型定方案，本地模型实施，达到触发条件才升级诊断。原功能与安全门禁在当前机上仍须满足，不预估人力工期。</t>
         </is>
       </c>
       <c r="B2" s="1" t="n"/>
@@ -1484,7 +1484,7 @@
     <row r="9" ht="27" customHeight="1">
       <c r="A9" s="61" t="inlineStr">
         <is>
-          <t>边界：50包含P00已完成成果归档，49包仍有剩余。6层=5条开工依赖边；原图20条边包含验收前置，两种口径不等于交付工期对比。新包状态不会因合并自动变完成。</t>
+          <t>边界：50包含P00已完成成果归档，P14另已单机验收，48包仍需推进。6层=5条开工依赖边；原图20条边包含验收前置，两种口径不等于交付工期对比。新包状态不会因合并自动变完成。</t>
         </is>
       </c>
       <c r="B9" s="1" t="n"/>
@@ -1530,7 +1530,7 @@
     <row r="12" ht="30" customHeight="1">
       <c r="A12" s="63" t="inlineStr">
         <is>
-          <t>当前执行模式：1 个 Root Worker 编排 + 最多 3 个写入子智能体。P14 在共同基线与共享合同冻结后，一次性并行派发 WEB/T041、CONTROL/版本固定与回退、ANDROID/下载激活与旧版保留；全部派发后再统一等待，禁止 spawn 一个就 await 一个。等待设备、授权或合同的空槽立即从 READY 池补位。</t>
+          <t>当前执行模式：Root + 最多3个隔离写入子智能体；P14 WEB/CONTROL/ANDROID已合并并完成OnePlus单机版本生命周期验收。当前继续按READY规则安排P09/G3检查及P15等独立模块，设备/部署仍单队列。</t>
         </is>
       </c>
       <c r="B12" s="1" t="n"/>
@@ -1548,7 +1548,7 @@
     <row r="13" ht="26" customHeight="1">
       <c r="A13" s="98" t="inlineStr">
         <is>
-          <t>启用前置：当前仓库只有一个脏 worktree，约 84 个已跟踪修改和 77 个未跟踪路径；不得直接多写者共享目录。Root Worker 先审核并建立可恢复集成基线，再为三个子智能体创建独立 worktree。开发可并行；共享合同、数据库迁移、主线合并、首尔部署、人工 Recipe 发布、OnePlus b0644fb5 真机写操作和 G3 副作用保持单队列。P14 未完整闭环前仍不启动 P15。</t>
+          <t>2026-09-10：集成分支 integration/p14-20260909，P14运行修复80a5de9/1ca0c1a，设备故障测试033e5ac/5eaa2f1。已建立独立worktree；不再重复WAIT_BASELINE。P14已解锁P15，但P15及G3尚未验收。</t>
         </is>
       </c>
       <c r="B13" s="1" t="n"/>
@@ -2973,22 +2973,52 @@
       </c>
     </row>
     <row r="15" ht="32" customHeight="1">
-      <c r="A15" s="92" t="n"/>
-      <c r="B15" s="92" t="n"/>
-      <c r="C15" s="92" t="n"/>
-      <c r="D15" s="92" t="n"/>
-      <c r="E15" s="92" t="n"/>
+      <c r="A15" s="92" t="inlineStr">
+        <is>
+          <t>R20260910-P14-01</t>
+        </is>
+      </c>
+      <c r="B15" s="92" t="inlineStr">
+        <is>
+          <t>P14</t>
+        </is>
+      </c>
+      <c r="C15" s="92" t="inlineStr">
+        <is>
+          <t>签名版本生命周期单机验收及等待/恢复修复</t>
+        </is>
+      </c>
+      <c r="D15" s="92" t="inlineStr">
+        <is>
+          <t>Codex Root + lamda-astra-worker×2</t>
+        </is>
+      </c>
+      <c r="E15" s="92" t="inlineStr">
+        <is>
+          <t>执行</t>
+        </is>
+      </c>
       <c r="F15" s="96" t="n"/>
-      <c r="G15" s="96" t="n"/>
+      <c r="G15" s="96" t="n">
+        <v>46275.03904717639</v>
+      </c>
       <c r="H15" s="92" t="n"/>
       <c r="I15" s="92" t="n"/>
       <c r="J15" s="92" t="n"/>
       <c r="K15" s="92" t="n"/>
       <c r="L15" s="92" t="n"/>
       <c r="M15" s="97" t="n"/>
-      <c r="N15" s="92" t="n"/>
+      <c r="N15" s="92" t="inlineStr">
+        <is>
+          <t>功能验收通过</t>
+        </is>
+      </c>
       <c r="O15" s="92" t="n"/>
-      <c r="P15" s="92" t="n"/>
+      <c r="P15" s="92" t="inlineStr">
+        <is>
+          <t>cloudctl-source/artifacts/tasks/P14-multi-agent/P14-INTEGRATION-ACCEPTANCE/summary.md；成本/Token未提供，留空。P09/G3与P15未验收。</t>
+        </is>
+      </c>
     </row>
     <row r="16" ht="32" customHeight="1">
       <c r="A16" s="91" t="n"/>
@@ -38905,7 +38935,7 @@
       </c>
       <c r="C5" s="90" t="inlineStr">
         <is>
-          <t>P14 Root Worker 多智能体并行交接（2026-09-09）</t>
+          <t>P14验收完成与后续接续（2026-09-10）</t>
         </is>
       </c>
     </row>
@@ -38922,7 +38952,7 @@
       </c>
       <c r="C6" s="91" t="inlineStr">
         <is>
-          <t>目标不变：P14 版本生命周期余项。执行拓扑改为 Root + 3 子智能体。当前仓库是单个脏 worktree，未形成共同基线前只允许并行只读分析；写入派发状态为 WAIT_BASELINE。</t>
+          <t>P14单机验收已完成；integration/p14-20260909含80a5de9、1ca0c1a、033e5ac、5eaa2f1。详见cloudctl-source/artifacts/tasks/P14-multi-agent/P14-INTEGRATION-ACCEPTANCE/summary.md</t>
         </is>
       </c>
     </row>
@@ -38939,7 +38969,7 @@
       </c>
       <c r="C7" s="92" t="inlineStr">
         <is>
-          <t>复用已关闭的签名安装、claim、WRONG_ACTIVE 与焦点硬验收；不重复 probe。共享输入由 Root 冻结为 recipe-version 合同/fixture；三路从同一基线 SHA 派生。</t>
+          <t>复用62 Android单测、3 OnePlus故障测试及真实签名版本发布/暂停/回退/HTTPS截断记录，不重做焦点probe。</t>
         </is>
       </c>
     </row>
@@ -38973,7 +39003,7 @@
       </c>
       <c r="C9" s="92" t="inlineStr">
         <is>
-          <t>Root 先审核当前 84 个已跟踪修改和 77 个未跟踪路径，排除缓存/二进制/SQLite/WAL/密钥后建立可恢复基线；再创建三个 worktree 并同批派发。不得 git add -A。</t>
+          <t>本轮修复wait空实现、等待状态恢复校验及设备测试目录；代码已提交。下一包按实际接口与验收缺口选取，不回到脏工作区基线步骤。</t>
         </is>
       </c>
     </row>
@@ -38990,7 +39020,7 @@
       </c>
       <c r="C10" s="91" t="inlineStr">
         <is>
-          <t>每个子智能体只需完成自身模块契约与测试；整包仍需 Root 在同一 integration SHA 上验证网页人工发布、签名版本 claim/执行、运行/暂停固定、断点下载、回退和审计。</t>
+          <t>P14验收矩阵已满足；P08仅同任务恢复检查点通过，P09/G3与P15分别验收。</t>
         </is>
       </c>
     </row>
@@ -39024,7 +39054,7 @@
       </c>
       <c r="C12" s="91" t="inlineStr">
         <is>
-          <t>三路开发并行；Control→Android→Web 是受控合并顺序，不是开发等待顺序。P14 等锁时可调度 P08/P16/P40/P48 的无冲突 READY 工作；P15 仍禁止启动。</t>
+          <t>P14依赖已解锁；设备active1.0.1、pending=null、最终c8ec815c探针成功。没有本轮运行/暂停任务，临时Nginx规则和故障服务已清理。</t>
         </is>
       </c>
     </row>
@@ -39075,7 +39105,7 @@
       </c>
       <c r="C15" s="92" t="inlineStr">
         <is>
-          <t>当前可执行的机器清单与 P14 队列见 11 表。运行时若不支持真实子智能体，明确报告能力缺失，不得用 Temporal Child Workflow 或普通串行函数冒充。</t>
+          <t>后续以本次单机验收报告为基线；公开Basic Auth登录未验证，G3真实业务提交门禁仍未通过。</t>
         </is>
       </c>
     </row>
@@ -39132,7 +39162,7 @@
     <row r="2" ht="42" customHeight="1">
       <c r="A2" s="112" t="inlineStr">
         <is>
-          <t>开发层：1个Root Worker + 最多3个写入子智能体；同轮先全部派发再统一等待。生产Temporal Worker不是LLM调度器。当前多写者启动前置=WAIT_BASELINE。</t>
+          <t>开发层：Root + 最多3个隔离写入子智能体。P14三路及集成单机验收已完成；不再WAIT_BASELINE。生产Temporal Worker不是LLM调度器。</t>
         </is>
       </c>
       <c r="B2" s="1" t="n"/>
@@ -39146,6 +39176,7 @@
       <c r="J2" s="1" t="n"/>
       <c r="K2" s="1" t="n"/>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="113" t="inlineStr">
         <is>
@@ -39272,7 +39303,7 @@
       </c>
       <c r="E8" s="115" t="inlineStr">
         <is>
-          <t>不启动P15、不扩二期</t>
+          <t>P15依赖已解锁；按READY安排，不扩二期</t>
         </is>
       </c>
       <c r="F8" s="115" t="inlineStr">
@@ -39609,7 +39640,7 @@
       </c>
       <c r="C26" s="119" t="inlineStr">
         <is>
-          <t>WAIT_BASELINE</t>
+          <t>COMPLETE</t>
         </is>
       </c>
       <c r="D26" s="119" t="inlineStr">
@@ -39666,7 +39697,7 @@
       </c>
       <c r="C27" s="119" t="inlineStr">
         <is>
-          <t>WAIT_BASELINE</t>
+          <t>ACCEPTED</t>
         </is>
       </c>
       <c r="D27" s="119" t="inlineStr">
@@ -39723,7 +39754,7 @@
       </c>
       <c r="C28" s="119" t="inlineStr">
         <is>
-          <t>WAIT_BASELINE</t>
+          <t>ACCEPTED</t>
         </is>
       </c>
       <c r="D28" s="119" t="inlineStr">
@@ -39780,7 +39811,7 @@
       </c>
       <c r="C29" s="119" t="inlineStr">
         <is>
-          <t>WAIT_BASELINE</t>
+          <t>ACCEPTED</t>
         </is>
       </c>
       <c r="D29" s="119" t="inlineStr">
@@ -39837,7 +39868,7 @@
       </c>
       <c r="C30" s="118" t="inlineStr">
         <is>
-          <t>WAIT_CHILDREN</t>
+          <t>ACCEPTED</t>
         </is>
       </c>
       <c r="D30" s="118" t="inlineStr">
@@ -40988,7 +41019,7 @@
       </c>
       <c r="D14" s="22" t="inlineStr">
         <is>
-          <t>已有实现待联调</t>
+          <t>核心通过</t>
         </is>
       </c>
       <c r="E14" s="22" t="inlineStr">
@@ -41033,7 +41064,7 @@
       </c>
       <c r="N14" s="100" t="inlineStr">
         <is>
-          <t>T026暂停握手 OnePlus 已过；ResumeValidator已接入。同taskId、CommandV1 领取后的续跑仍待真机验收。不重写已通过握手。真实副作用仍须G3。</t>
+          <t>2026-09-10：caa22da3 CommandV1签名任务，PAUSED_WAITING_USER后保留数据安装APK，原taskId恢复RUNNING，resumeCount=2，保持1.0.3并从hold继续，started未重放；pageVerified=false拒绝409。取证后主动取消。其他G2故障不据此自动通过。见 cloudctl-source/artifacts/tasks/P14-multi-agent/P14-INTEGRATION-ACCEPTANCE/summary.md</t>
         </is>
       </c>
       <c r="O14" s="4" t="inlineStr">
@@ -41057,7 +41088,7 @@
       </c>
       <c r="S14" s="100" t="inlineStr">
         <is>
-          <t>可用探针补一轮同taskId续跑；不要重写已通过握手。真实副作用仍须G3。当前验收机=OnePlus 9R b0644fb5。</t>
+          <t>同taskId续跑不再重复开发；后续补失租立停等G2故障，P09/G3真实副作用门禁仍未过。</t>
         </is>
       </c>
     </row>
@@ -41534,7 +41565,7 @@
       </c>
       <c r="D20" s="22" t="inlineStr">
         <is>
-          <t>进行中</t>
+          <t>验收通过</t>
         </is>
       </c>
       <c r="E20" s="22" t="inlineStr">
@@ -41574,12 +41605,12 @@
       </c>
       <c r="M20" s="22" t="inlineStr">
         <is>
-          <t>部分可用</t>
+          <t>可用</t>
         </is>
       </c>
       <c r="N20" s="100" t="inlineStr">
         <is>
-          <t>2026-09-09：签名 Recipe 1.0.1（825921a4…，phase1-recipe-1）已人工发布，并由 OnePlus 9R 自动下载、验签安装；签名校验保持开启。焦点硬验收任务 0d36fe3f… 在闲鱼前台起始时 SUCCEEDED attempt=1，日志证明 launchTargetApp 等待后 expected=actual=Companion；历史任务 7f292679 仍 FAILED/WRONG_ACTIVE_PACKAGE。该硬验收执行的是内置 Recipe 901f795b…，不能作为签名 Recipe 被 claim 固定并执行的证据。后端相关 6 项测试通过，Android Recipe 定向测试 BUILD SUCCESSFUL。未完成：T041 网页人工发布入口、签名版本任务固定/执行、运行及暂停任务固定旧版、下载中断保留旧版、真实回退与每设备版本审计。</t>
+          <t>2026-09-10 OnePlus单机验收通过：网页人工登记/发布/回退；签名版本真实领取执行；caa22da3同任务运行中发布新版、暂停、APK重启、恢复均固定1.0.3且不重放已完成步；真实HTTPS 685→32字节截断时保留1.0.1，恢复后自动验签激活1.0.4；最后回退1.0.1并由c8ec815c探针成功。62 Android单测、3真机存储故障测试通过。见 cloudctl-source/artifacts/tasks/P14-multi-agent/P14-INTEGRATION-ACCEPTANCE/summary.md</t>
         </is>
       </c>
       <c r="O20" s="4" t="inlineStr">
@@ -41593,17 +41624,17 @@
       </c>
       <c r="Q20" s="22" t="inlineStr">
         <is>
-          <t>开发中</t>
+          <t>模块通过</t>
         </is>
       </c>
       <c r="R20" s="22" t="inlineStr">
         <is>
-          <t>WAIT_BASELINE</t>
+          <t>无</t>
         </is>
       </c>
       <c r="S20" s="100" t="inlineStr">
         <is>
-          <t>短前置：Root 审核当前脏工作区并冻结共同 SHA/recipe-version 合同。随后同批启动 P14-WEB-T041、P14-CONTROL-VERSION、P14-ANDROID-LIFECYCLE 三路；等待锁时用 P08/P16/P40/P48 的 READY 工作补槽。三路开发完成后由 Root 按 Control→Android→Web 合并并统一生成合同；设备/发布验收单队列。P14 通过前不启动 P15。</t>
+          <t>P14依赖已解锁；允许按READY规则安排P15。P08同任务恢复已补证，其他G2故障及P09/G3仍需独立验收。公网Basic Auth登录未计入本次通过范围。</t>
         </is>
       </c>
     </row>
@@ -45550,7 +45581,7 @@
       </c>
       <c r="C20" s="101" t="inlineStr">
         <is>
-          <t>2026-09-09 焦点硬验收已通过：0d36fe3f… 从闲鱼前台起始，执行器等待后 expected/actual 均为 Companion；7f292679 保持历史失败。签名包 825921a4… 已下载验签安装，但本次 probe 使用内置 901f795b…，尚未证明已发布签名版本被任务固定并执行。下一步只做版本生命周期余项，不重复焦点 probe，不启动 P15。</t>
+          <t>2026-09-10 单机签名版本生命周期验收通过，详见 cloudctl-source/artifacts/tasks/P14-multi-agent/P14-INTEGRATION-ACCEPTANCE/summary.md。P15依赖已解锁，G3仍未过。</t>
         </is>
       </c>
       <c r="D20" s="4" t="inlineStr">
@@ -48364,7 +48395,7 @@
       </c>
       <c r="D34" s="4" t="inlineStr">
         <is>
-          <t>P14 焦点硬验收已通过；当前优先完成 P14 版本生命周期余项，并保持 P08 CommandV1 同 task 续跑待验。P14 未闭环前不启动 P15；不从新基线重跑。</t>
+          <t>2026-09-10：P14单机版本生命周期通过，P08同task恢复已补证。下一步核对P09/G3故障矩阵，可按READY安排P15。不得扩记其他包完成。</t>
         </is>
       </c>
       <c r="E34" s="4" t="inlineStr">

</xml_diff>

<commit_message>
Verify P09 guards on OnePlus and record remaining commit wiring
</commit_message>
<xml_diff>
--- a/docs/project-plans/lamda_yun_一期计划_智能体执行版.xlsx
+++ b/docs/project-plans/lamda_yun_一期计划_智能体执行版.xlsx
@@ -3000,7 +3000,7 @@
       </c>
       <c r="F15" s="96" t="n"/>
       <c r="G15" s="96" t="n">
-        <v>46275.03904717639</v>
+        <v>46275.03904717592</v>
       </c>
       <c r="H15" s="92" t="n"/>
       <c r="I15" s="92" t="n"/>
@@ -3021,22 +3021,52 @@
       </c>
     </row>
     <row r="16" ht="32" customHeight="1">
-      <c r="A16" s="91" t="n"/>
-      <c r="B16" s="91" t="n"/>
-      <c r="C16" s="91" t="n"/>
-      <c r="D16" s="91" t="n"/>
-      <c r="E16" s="91" t="n"/>
+      <c r="A16" s="91" t="inlineStr">
+        <is>
+          <t>R20260910-P09-01</t>
+        </is>
+      </c>
+      <c r="B16" s="91" t="inlineStr">
+        <is>
+          <t>P09</t>
+        </is>
+      </c>
+      <c r="C16" s="91" t="inlineStr">
+        <is>
+          <t>不确定状态保护与本地防重切片</t>
+        </is>
+      </c>
+      <c r="D16" s="91" t="inlineStr">
+        <is>
+          <t>Codex Root + lamda-astra-worker×2</t>
+        </is>
+      </c>
+      <c r="E16" s="91" t="inlineStr">
+        <is>
+          <t>执行</t>
+        </is>
+      </c>
       <c r="F16" s="94" t="n"/>
-      <c r="G16" s="94" t="n"/>
+      <c r="G16" s="94" t="n">
+        <v>46275.06336192244</v>
+      </c>
       <c r="H16" s="91" t="n"/>
       <c r="I16" s="91" t="n"/>
       <c r="J16" s="91" t="n"/>
       <c r="K16" s="91" t="n"/>
       <c r="L16" s="91" t="n"/>
       <c r="M16" s="95" t="n"/>
-      <c r="N16" s="91" t="n"/>
+      <c r="N16" s="91" t="inlineStr">
+        <is>
+          <t>模块通过</t>
+        </is>
+      </c>
       <c r="O16" s="91" t="n"/>
-      <c r="P16" s="91" t="n"/>
+      <c r="P16" s="91" t="inlineStr">
+        <is>
+          <t>cloudctl-source/artifacts/tasks/P09-unknown/hardening-20260910.md；G3未验收。调用成本未提供，留空。</t>
+        </is>
+      </c>
     </row>
     <row r="17" ht="32" customHeight="1">
       <c r="A17" s="92" t="n"/>
@@ -38935,7 +38965,7 @@
       </c>
       <c r="C5" s="90" t="inlineStr">
         <is>
-          <t>P14验收完成与后续接续（2026-09-10）</t>
+          <t>P09提交与核对链路接线（2026-09-10）</t>
         </is>
       </c>
     </row>
@@ -38952,7 +38982,7 @@
       </c>
       <c r="C6" s="91" t="inlineStr">
         <is>
-          <t>P14单机验收已完成；integration/p14-20260909含80a5de9、1ca0c1a、033e5ac、5eaa2f1。详见cloudctl-source/artifacts/tasks/P14-multi-agent/P14-INTEGRATION-ACCEPTANCE/summary.md</t>
+          <t>P14已单机验收；P09状态保护切片已部署，backend21202a5、Android ef9eb2b。当前继续P09真正提交链路，G3尚未通过。</t>
         </is>
       </c>
     </row>
@@ -38969,7 +38999,7 @@
       </c>
       <c r="C7" s="92" t="inlineStr">
         <is>
-          <t>复用62 Android单测、3 OnePlus故障测试及真实签名版本发布/暂停/回退/HTTPS截断记录，不重做焦点probe。</t>
+          <t>89后端、78Android、3真机本地计数测试与5897215f部署探针。复用ActionJournal、Coordinator和既有server reconcile，不重写已过的P14。</t>
         </is>
       </c>
     </row>
@@ -39003,7 +39033,7 @@
       </c>
       <c r="C9" s="92" t="inlineStr">
         <is>
-          <t>本轮修复wait空实现、等待状态恢复校验及设备测试目录；代码已提交。下一包按实际接口与验收缺口选取，不回到脏工作区基线步骤。</t>
+          <t>先冻结云端intent与本地once gate顺序、明确后置确认及服务端核对到手机的可信同步。现有CommitIntentRow绑定publish_target，禁止把mobile taskId伪装成targetId。</t>
         </is>
       </c>
     </row>
@@ -39020,7 +39050,7 @@
       </c>
       <c r="C10" s="91" t="inlineStr">
         <is>
-          <t>P14验收矩阵已满足；P08仅同任务恢复检查点通过，P09/G3与P15分别验收。</t>
+          <t>状态加固模块通过；下一切片需云端/本地一次提交与恢复测试。未进行真实平台副作用，G3不得记完成。</t>
         </is>
       </c>
     </row>
@@ -39054,7 +39084,7 @@
       </c>
       <c r="C12" s="91" t="inlineStr">
         <is>
-          <t>P14依赖已解锁；设备active1.0.1、pending=null、最终c8ec815c探针成功。没有本轮运行/暂停任务，临时Nginx规则和故障服务已清理。</t>
+          <t>当前生产Recipe尚未调用独立IrreversibleActionCoordinator。真实商品不用于代码调试，先用独立测试数据。Root继续独占设备、部署和最终验收。</t>
         </is>
       </c>
     </row>
@@ -39105,7 +39135,7 @@
       </c>
       <c r="C15" s="92" t="inlineStr">
         <is>
-          <t>后续以本次单机验收报告为基线；公开Basic Auth登录未验证，G3真实业务提交门禁仍未通过。</t>
+          <t>cloudctl-source/artifacts/tasks/P09-unknown/hardening-20260910.md；下一契约参考同目录next-integration-slice.md。</t>
         </is>
       </c>
     </row>
@@ -41110,7 +41140,7 @@
       </c>
       <c r="D15" s="22" t="inlineStr">
         <is>
-          <t>已有实现待联调</t>
+          <t>进行中</t>
         </is>
       </c>
       <c r="E15" s="22" t="inlineStr">
@@ -41155,7 +41185,7 @@
       </c>
       <c r="N15" s="100" t="inlineStr">
         <is>
-          <t>action_journal单测 + 007 SQL已有；UNKNOWN/终态门禁已接。无真机断网二次提交。G3未过。禁止真发布/鱼币/删除。</t>
+          <t>2026-09-10 已加固并部署RECONCILING双端状态保护：普通完成/暂停/取消/恢复不得清除UNKNOWN；Android默认未确认不记APPLIED，重启/续租/新任务不得绕过。89后端测试、78Android单测、3OnePlus独立计数故障测试通过，部署后5897215f探针成功。G3未通过：仍缺真实Recipe提交接线、云端intent与双端核对同步。见 cloudctl-source/artifacts/tasks/P09-unknown/hardening-20260910.md</t>
         </is>
       </c>
       <c r="O15" s="4" t="inlineStr">
@@ -41174,12 +41204,12 @@
       </c>
       <c r="R15" s="22" t="inlineStr">
         <is>
-          <t>待核实</t>
+          <t>无</t>
         </is>
       </c>
       <c r="S15" s="100" t="inlineStr">
         <is>
-          <t>高风险动作继续共用本门禁；G3前禁止真发布/鱼币/删除。不得把模块通过当成 G3 已过。</t>
+          <t>下一切片冻结提交前记账、一次执行、后置结果与核对同步契约；完成无副作用闭环后再确定各真实动作的测试对象/预算。不得把本地计数当真实G3通过。</t>
         </is>
       </c>
     </row>
@@ -45371,7 +45401,7 @@
       </c>
       <c r="C15" s="101" t="inlineStr">
         <is>
-          <t>UNKNOWN/终态门禁已接。G3前不跑真实发布、鱼币或删除。</t>
+          <t>双端RECONCILING加固已部署，89后端/78Android/3设备计数测试通过。真实提交接线与G3仍待验，见 cloudctl-source/artifacts/tasks/P09-unknown/hardening-20260910.md</t>
         </is>
       </c>
       <c r="D15" s="4" t="inlineStr">

</xml_diff>